<commit_message>
Made some changes to mock data
</commit_message>
<xml_diff>
--- a/Mock_NYP2025-001_Campaign_Master.xlsx
+++ b/Mock_NYP2025-001_Campaign_Master.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CHAN GILBERT\Documents\My Tableau Repository\Datasources\2024.3\en_US-US\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\CETMarketingKiro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B904CE53-2FDA-4EA3-B4D3-07B623198437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD77A39B-FD8C-4CE3-A7A2-71DC51F15FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="1" activeTab="1" xr2:uid="{55593DBD-70AE-49DD-AF1D-992C0FB64303}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{55593DBD-70AE-49DD-AF1D-992C0FB64303}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="2" r:id="rId1"/>
     <sheet name="Master" sheetId="1" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Master!$A$1:$N$31</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -963,7 +966,7 @@
     <col min="4" max="4" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" customWidth="1"/>
     <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="32" bestFit="1" customWidth="1"/>
@@ -1435,7 +1438,7 @@
         <v>45424</v>
       </c>
       <c r="H11" s="1">
-        <v>45459</v>
+        <v>45453</v>
       </c>
       <c r="I11" t="s">
         <v>37</v>
@@ -1783,10 +1786,10 @@
       <c r="F19" t="s">
         <v>14</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <v>45295</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="1">
         <v>45310</v>
       </c>
       <c r="I19" t="s">
@@ -1827,11 +1830,11 @@
       <c r="F20" t="s">
         <v>14</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <v>45295</v>
       </c>
-      <c r="H20">
-        <v>45310</v>
+      <c r="H20" s="1">
+        <v>45301</v>
       </c>
       <c r="I20" t="s">
         <v>31</v>
@@ -2289,6 +2292,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N31" xr:uid="{0B272666-4372-4ACB-8063-01DE39C797EF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Calibri"&amp;10&amp;K000000 Official (Closed) and Sensitive-Normal&amp;1#_x000D_</oddHeader>

</xml_diff>